<commit_message>
feat(utility): un-stub standalone workflows and add MSMS domain
- Implement get_or_create_utility_environment for standalone fallback
- Port document converters into src/postprocessing domain package
- Un-stub all 11 standalone utility action runners in utility_actions.py
- Add 1-Click Substation Post-Processing Pipeline workflow
- Add src/msms domain package and update_data_msms workflow for WO sync
- All 73 test cases passing cleanly
</commit_message>
<xml_diff>
--- a/templates/DATA MSMS.xlsx
+++ b/templates/DATA MSMS.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADAM\Documents\PO 42234207 - JOHOR - JBU - 400 PE IR US TEV\PYTHON\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADAM\Desktop\pahang-cli\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC36E9D9-A0B2-4A34-BCD5-5049B50E5950}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63CB91F0-70C5-4412-9DB6-CAFAE9D9B0D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="316">
   <si>
     <t>Work Order</t>
   </si>
@@ -63,6 +63,924 @@
   </si>
   <si>
     <t>S/S WBT.48 K.TERLA</t>
+  </si>
+  <si>
+    <t>W1544480</t>
+  </si>
+  <si>
+    <t>CKTN/PCEJ00021</t>
+  </si>
+  <si>
+    <t>SEK MEN GUDANG RASAU</t>
+  </si>
+  <si>
+    <t>W1545091</t>
+  </si>
+  <si>
+    <t>CKTN/PCEJ01071</t>
+  </si>
+  <si>
+    <t>PASARAYA HAPPY HOME</t>
+  </si>
+  <si>
+    <t>W1545123</t>
+  </si>
+  <si>
+    <t>CKTN/PCEJ01118</t>
+  </si>
+  <si>
+    <t>TAMAN TAS RIA 2 LOT 2368</t>
+  </si>
+  <si>
+    <t>W1545168</t>
+  </si>
+  <si>
+    <t>CKTN/PCEJ01208</t>
+  </si>
+  <si>
+    <t>TAMAN AZLINA</t>
+  </si>
+  <si>
+    <t>W1545225</t>
+  </si>
+  <si>
+    <t>CKTN/PCEJ01334</t>
+  </si>
+  <si>
+    <t>TAMAN SRI DAMAI PERDANA</t>
+  </si>
+  <si>
+    <t>W1545277</t>
+  </si>
+  <si>
+    <t>CKTN/PCEJ01439</t>
+  </si>
+  <si>
+    <t>PE KEDAI DAMAI PERDANA</t>
+  </si>
+  <si>
+    <t>W1544478</t>
+  </si>
+  <si>
+    <t>CKTN/PCEJ00018</t>
+  </si>
+  <si>
+    <t>KEDAI TAMAN GURU</t>
+  </si>
+  <si>
+    <t>W1544997</t>
+  </si>
+  <si>
+    <t>CKTN/PCEJ00869</t>
+  </si>
+  <si>
+    <t>TMN ANEKA JAYA LOT 984</t>
+  </si>
+  <si>
+    <t>W1544476</t>
+  </si>
+  <si>
+    <t>CKTN/PCEJ00014</t>
+  </si>
+  <si>
+    <t>SEK KEB KAMPUNG PANDAN</t>
+  </si>
+  <si>
+    <t>W1544479</t>
+  </si>
+  <si>
+    <t>CKTN/PCEJ00019</t>
+  </si>
+  <si>
+    <t>BALAI BOMBA TAMAN TAS</t>
+  </si>
+  <si>
+    <t>W1544509</t>
+  </si>
+  <si>
+    <t>CKTN/PCEJ00074</t>
+  </si>
+  <si>
+    <t>KUARTERS GURU SEK KEB PANDAN</t>
+  </si>
+  <si>
+    <t>W1545035</t>
+  </si>
+  <si>
+    <t>CKTN/PCEJ00962</t>
+  </si>
+  <si>
+    <t>LOT 26658 KTN BYPASS SENG KEE</t>
+  </si>
+  <si>
+    <t>W1545199</t>
+  </si>
+  <si>
+    <t>CKTN/PCEJ01296</t>
+  </si>
+  <si>
+    <t>TAS DAGANGAN 1</t>
+  </si>
+  <si>
+    <t>W1545222</t>
+  </si>
+  <si>
+    <t>CKTN/PCEJ01331</t>
+  </si>
+  <si>
+    <t>PERWIRA PANDAN</t>
+  </si>
+  <si>
+    <t>W1545335</t>
+  </si>
+  <si>
+    <t>CKTN/PCEJ01542</t>
+  </si>
+  <si>
+    <t>ANEKA JAYA 82</t>
+  </si>
+  <si>
+    <t>W1545565</t>
+  </si>
+  <si>
+    <t>CKTN/PCEJ01719</t>
+  </si>
+  <si>
+    <t>CS PETRON PANDAN (KTN 4577)</t>
+  </si>
+  <si>
+    <t>W1547841</t>
+  </si>
+  <si>
+    <t>CCHL/PCEJ00002</t>
+  </si>
+  <si>
+    <t>JALAN ROBINSON</t>
+  </si>
+  <si>
+    <t>W1547904</t>
+  </si>
+  <si>
+    <t>CCHL/PCEJ00124</t>
+  </si>
+  <si>
+    <t>HABU HEIGHT</t>
+  </si>
+  <si>
+    <t>W1547963</t>
+  </si>
+  <si>
+    <t>CCHL/PCEJ00233</t>
+  </si>
+  <si>
+    <t>KG.ASLI TEJI</t>
+  </si>
+  <si>
+    <t>W1547985</t>
+  </si>
+  <si>
+    <t>CCHL/PCEJ00261</t>
+  </si>
+  <si>
+    <t>PINANG &amp; TIAT</t>
+  </si>
+  <si>
+    <t>W1547986</t>
+  </si>
+  <si>
+    <t>CCHL/PCEJ00262</t>
+  </si>
+  <si>
+    <t>KG. SUSU</t>
+  </si>
+  <si>
+    <t>W1547852</t>
+  </si>
+  <si>
+    <t>CCHL/PCEJ00024</t>
+  </si>
+  <si>
+    <t>GAONG SHANG ULU BERTAM</t>
+  </si>
+  <si>
+    <t>W1547853</t>
+  </si>
+  <si>
+    <t>CCHL/PCEJ00025</t>
+  </si>
+  <si>
+    <t>BERTAM FARM</t>
+  </si>
+  <si>
+    <t>W1547854</t>
+  </si>
+  <si>
+    <t>CCHL/PCEJ00026</t>
+  </si>
+  <si>
+    <t>POH HUAT FARM,ULU BERTAM</t>
+  </si>
+  <si>
+    <t>W1547855</t>
+  </si>
+  <si>
+    <t>CCHL/PCEJ00027</t>
+  </si>
+  <si>
+    <t>PALACE ROSE</t>
+  </si>
+  <si>
+    <t>W1547869</t>
+  </si>
+  <si>
+    <t>CCHL/PCEJ00052</t>
+  </si>
+  <si>
+    <t>SUNLIGHT FARM</t>
+  </si>
+  <si>
+    <t>W1547909</t>
+  </si>
+  <si>
+    <t>CCHL/PCEJ00132</t>
+  </si>
+  <si>
+    <t>KHOR LENG HUAT</t>
+  </si>
+  <si>
+    <t>W1547945</t>
+  </si>
+  <si>
+    <t>CCHL/PCEJ00206</t>
+  </si>
+  <si>
+    <t>KG ASLI SUNGAI KABOK</t>
+  </si>
+  <si>
+    <t>W1547956</t>
+  </si>
+  <si>
+    <t>CCHL/PCEJ00223</t>
+  </si>
+  <si>
+    <t>KG ASLI KUALA BOH</t>
+  </si>
+  <si>
+    <t>W1547960</t>
+  </si>
+  <si>
+    <t>CCHL/PCEJ00228</t>
+  </si>
+  <si>
+    <t>KG ASLI RELONG</t>
+  </si>
+  <si>
+    <t>W1547962</t>
+  </si>
+  <si>
+    <t>CCHL/PCEJ00231</t>
+  </si>
+  <si>
+    <t>TAN BUEY TEK</t>
+  </si>
+  <si>
+    <t>W1547981</t>
+  </si>
+  <si>
+    <t>CCHL/PCEJ00256</t>
+  </si>
+  <si>
+    <t>PPRT LEMBAH BERTAM</t>
+  </si>
+  <si>
+    <t>W1547983</t>
+  </si>
+  <si>
+    <t>CCHL/PCEJ00258</t>
+  </si>
+  <si>
+    <t>LOT 201 MARDI</t>
+  </si>
+  <si>
+    <t>W1547850</t>
+  </si>
+  <si>
+    <t>CCHL/PCEJ00022</t>
+  </si>
+  <si>
+    <t>PE MOOI FOOK FARM</t>
+  </si>
+  <si>
+    <t>W1547851</t>
+  </si>
+  <si>
+    <t>CCHL/PCEJ00023</t>
+  </si>
+  <si>
+    <t>UNIVERSAL ULU BERTAM</t>
+  </si>
+  <si>
+    <t>W1547865</t>
+  </si>
+  <si>
+    <t>CCHL/PCEJ00041</t>
+  </si>
+  <si>
+    <t>NOTRE DAM BT.33</t>
+  </si>
+  <si>
+    <t>W1547890</t>
+  </si>
+  <si>
+    <t>CCHL/PCEJ00104</t>
+  </si>
+  <si>
+    <t>HEN CHIK HAN</t>
+  </si>
+  <si>
+    <t>W1547944</t>
+  </si>
+  <si>
+    <t>CCHL/PCEJ00204</t>
+  </si>
+  <si>
+    <t>SAL QUARY</t>
+  </si>
+  <si>
+    <t>W1547946</t>
+  </si>
+  <si>
+    <t>CCHL/PCEJ00207</t>
+  </si>
+  <si>
+    <t>KIN FOOK FARM</t>
+  </si>
+  <si>
+    <t>W1547954</t>
+  </si>
+  <si>
+    <t>CCHL/PCEJ00220</t>
+  </si>
+  <si>
+    <t>MAFC NO.1</t>
+  </si>
+  <si>
+    <t>W1547955</t>
+  </si>
+  <si>
+    <t>CCHL/PCEJ00221</t>
+  </si>
+  <si>
+    <t>PE MAFC 2</t>
+  </si>
+  <si>
+    <t>W1547972</t>
+  </si>
+  <si>
+    <t>CCHL/PCEJ00245</t>
+  </si>
+  <si>
+    <t>PE KREMATORIUM HINDU</t>
+  </si>
+  <si>
+    <t>W1546840</t>
+  </si>
+  <si>
+    <t>CRAU/PCEJ00099</t>
+  </si>
+  <si>
+    <t>SEM FONG</t>
+  </si>
+  <si>
+    <t>W1546841</t>
+  </si>
+  <si>
+    <t>CRAU/PCEJ00100</t>
+  </si>
+  <si>
+    <t>PERABUT</t>
+  </si>
+  <si>
+    <t>W1546842</t>
+  </si>
+  <si>
+    <t>CRAU/PCEJ00101</t>
+  </si>
+  <si>
+    <t>CHEROH</t>
+  </si>
+  <si>
+    <t>W1546844</t>
+  </si>
+  <si>
+    <t>CRAU/PCEJ00103</t>
+  </si>
+  <si>
+    <t>TAMAN AMALINA PERDANA</t>
+  </si>
+  <si>
+    <t>W1546852</t>
+  </si>
+  <si>
+    <t>CRAU/PCEJ00112</t>
+  </si>
+  <si>
+    <t>LOJI AIR SEMANTAN</t>
+  </si>
+  <si>
+    <t>W1546853</t>
+  </si>
+  <si>
+    <t>CRAU/PCEJ00113</t>
+  </si>
+  <si>
+    <t>TAMAN BINTANG</t>
+  </si>
+  <si>
+    <t>W1546954</t>
+  </si>
+  <si>
+    <t>CRAU/PCEJ00258</t>
+  </si>
+  <si>
+    <t>LAMAN PESONA CHEROH</t>
+  </si>
+  <si>
+    <t>W1546961</t>
+  </si>
+  <si>
+    <t>CRAU/PCEJ00265</t>
+  </si>
+  <si>
+    <t>TAMAN PASDEC</t>
+  </si>
+  <si>
+    <t>W1546901</t>
+  </si>
+  <si>
+    <t>CRAU/PCEJ00172</t>
+  </si>
+  <si>
+    <t>SEK MEN TERSANG</t>
+  </si>
+  <si>
+    <t>W1546902</t>
+  </si>
+  <si>
+    <t>CRAU/PCEJ00173</t>
+  </si>
+  <si>
+    <t>FELDA TERSANG 1</t>
+  </si>
+  <si>
+    <t>W1546903</t>
+  </si>
+  <si>
+    <t>CRAU/PCEJ00174</t>
+  </si>
+  <si>
+    <t>BOOSTER TERSANG</t>
+  </si>
+  <si>
+    <t>W1546937</t>
+  </si>
+  <si>
+    <t>CRAU/PCEJ00231</t>
+  </si>
+  <si>
+    <t>KOLAM IKAN TERSANG</t>
+  </si>
+  <si>
+    <t>W1546953</t>
+  </si>
+  <si>
+    <t>CRAU/PCEJ00252</t>
+  </si>
+  <si>
+    <t>LADANG KREATIF</t>
+  </si>
+  <si>
+    <t>W1546976</t>
+  </si>
+  <si>
+    <t>CRAU/PCEJ00287</t>
+  </si>
+  <si>
+    <t>PE PGBF KOYAN 1</t>
+  </si>
+  <si>
+    <t>W1546906</t>
+  </si>
+  <si>
+    <t>CRAU/PCEJ00195</t>
+  </si>
+  <si>
+    <t>FELDA KOYAN 3</t>
+  </si>
+  <si>
+    <t>W1546907</t>
+  </si>
+  <si>
+    <t>CRAU/PCEJ00196</t>
+  </si>
+  <si>
+    <t>FELDA KOYAN 3 BARU</t>
+  </si>
+  <si>
+    <t>W1546949</t>
+  </si>
+  <si>
+    <t>CRAU/PCEJ00248</t>
+  </si>
+  <si>
+    <t>KG ASLI PANTOS</t>
+  </si>
+  <si>
+    <t>W1546968</t>
+  </si>
+  <si>
+    <t>CRAU/PCEJ00272</t>
+  </si>
+  <si>
+    <t>KG. TELOM</t>
+  </si>
+  <si>
+    <t>W1546876</t>
+  </si>
+  <si>
+    <t>CRAU/PCEJ00137</t>
+  </si>
+  <si>
+    <t>SUNGAI LIPAN</t>
+  </si>
+  <si>
+    <t>W1546877</t>
+  </si>
+  <si>
+    <t>CRAU/PCEJ00138</t>
+  </si>
+  <si>
+    <t>RM JERAM BESU</t>
+  </si>
+  <si>
+    <t>W1546878</t>
+  </si>
+  <si>
+    <t>CRAU/PCEJ00139</t>
+  </si>
+  <si>
+    <t>JERAM BESU</t>
+  </si>
+  <si>
+    <t>W1546883</t>
+  </si>
+  <si>
+    <t>CRAU/PCEJ00147</t>
+  </si>
+  <si>
+    <t>SEGA</t>
+  </si>
+  <si>
+    <t>W1546884</t>
+  </si>
+  <si>
+    <t>CRAU/PCEJ00148</t>
+  </si>
+  <si>
+    <t>ULU RENGGOL</t>
+  </si>
+  <si>
+    <t>W1546885</t>
+  </si>
+  <si>
+    <t>CRAU/PCEJ00151</t>
+  </si>
+  <si>
+    <t>DESA SEGA</t>
+  </si>
+  <si>
+    <t>W1546910</t>
+  </si>
+  <si>
+    <t>CRAU/PCEJ00199</t>
+  </si>
+  <si>
+    <t>VCB STATION TAMAN DONG JAYA</t>
+  </si>
+  <si>
+    <t>W1546958</t>
+  </si>
+  <si>
+    <t>CRAU/PCEJ00262</t>
+  </si>
+  <si>
+    <t>TAMAN DONG JAYA</t>
+  </si>
+  <si>
+    <t>W1546975</t>
+  </si>
+  <si>
+    <t>CRAU/PCEJ00283</t>
+  </si>
+  <si>
+    <t>PE CHICKEN COOP</t>
+  </si>
+  <si>
+    <t>W1546766</t>
+  </si>
+  <si>
+    <t>CRAU/PCEJ00001</t>
+  </si>
+  <si>
+    <t>RM BUKIT KOMAN</t>
+  </si>
+  <si>
+    <t>W1546767</t>
+  </si>
+  <si>
+    <t>CRAU/PCEJ00002</t>
+  </si>
+  <si>
+    <t>BUKIT KOMAN</t>
+  </si>
+  <si>
+    <t>W1546941</t>
+  </si>
+  <si>
+    <t>CRAU/PCEJ00235</t>
+  </si>
+  <si>
+    <t>RAUB OIL MILL S/B</t>
+  </si>
+  <si>
+    <t>W1546985</t>
+  </si>
+  <si>
+    <t>CRAU/PCEJ00309</t>
+  </si>
+  <si>
+    <t>SSU RAUB KOMERSIL</t>
+  </si>
+  <si>
+    <t>W1546900</t>
+  </si>
+  <si>
+    <t>CRAU/PCEJ00169</t>
+  </si>
+  <si>
+    <t>SIMPANG TERSANG</t>
+  </si>
+  <si>
+    <t>W1547892</t>
+  </si>
+  <si>
+    <t>CCHL/PCEJ00108</t>
+  </si>
+  <si>
+    <t>KUALA TERLA</t>
+  </si>
+  <si>
+    <t>W1547900</t>
+  </si>
+  <si>
+    <t>CCHL/PCEJ00119</t>
+  </si>
+  <si>
+    <t>DESA CORINA</t>
+  </si>
+  <si>
+    <t>W1547902</t>
+  </si>
+  <si>
+    <t>CCHL/PCEJ00121</t>
+  </si>
+  <si>
+    <t>TAMAN PINGGIRAN TERLA</t>
+  </si>
+  <si>
+    <t>W1547931</t>
+  </si>
+  <si>
+    <t>CCHL/PCEJ00174</t>
+  </si>
+  <si>
+    <t>PANGSAPURI FANTASIA</t>
+  </si>
+  <si>
+    <t>W1547947</t>
+  </si>
+  <si>
+    <t>CCHL/PCEJ00208</t>
+  </si>
+  <si>
+    <t>OMNI CASSIA</t>
+  </si>
+  <si>
+    <t>W1547961</t>
+  </si>
+  <si>
+    <t>CCHL/PCEJ00230</t>
+  </si>
+  <si>
+    <t>FABULAS GARDEN</t>
+  </si>
+  <si>
+    <t>W1547979</t>
+  </si>
+  <si>
+    <t>CCHL/PCEJ00253</t>
+  </si>
+  <si>
+    <t>PE VARIASI VILLA</t>
+  </si>
+  <si>
+    <t>W1547982</t>
+  </si>
+  <si>
+    <t>CCHL/PCEJ00257</t>
+  </si>
+  <si>
+    <t>OMNI CASSIA 2</t>
+  </si>
+  <si>
+    <t>W1547988</t>
+  </si>
+  <si>
+    <t>CCHL/PCEJ00267</t>
+  </si>
+  <si>
+    <t>NUOVOLAND</t>
+  </si>
+  <si>
+    <t>W1547870</t>
+  </si>
+  <si>
+    <t>CCHL/PCEJ00056</t>
+  </si>
+  <si>
+    <t>LIAN HING BATU 49</t>
+  </si>
+  <si>
+    <t>W1547897</t>
+  </si>
+  <si>
+    <t>CCHL/PCEJ00116</t>
+  </si>
+  <si>
+    <t>TRINGKAP</t>
+  </si>
+  <si>
+    <t>W1547898</t>
+  </si>
+  <si>
+    <t>CCHL/PCEJ00117</t>
+  </si>
+  <si>
+    <t>TRINGKAP PUNCAK 2</t>
+  </si>
+  <si>
+    <t>W1547899</t>
+  </si>
+  <si>
+    <t>CCHL/PCEJ00118</t>
+  </si>
+  <si>
+    <t>TRINGKAP PUNCAK 1</t>
+  </si>
+  <si>
+    <t>W1547936</t>
+  </si>
+  <si>
+    <t>CCHL/PCEJ00183</t>
+  </si>
+  <si>
+    <t>KHAW CHAI FATT</t>
+  </si>
+  <si>
+    <t>W1547939</t>
+  </si>
+  <si>
+    <t>CCHL/PCEJ00187</t>
+  </si>
+  <si>
+    <t>KG ASLI GETAN</t>
+  </si>
+  <si>
+    <t>W1547940</t>
+  </si>
+  <si>
+    <t>CCHL/PCEJ00188</t>
+  </si>
+  <si>
+    <t>KG ASLI TERLIMAU</t>
+  </si>
+  <si>
+    <t>W1547941</t>
+  </si>
+  <si>
+    <t>CCHL/PCEJ00189</t>
+  </si>
+  <si>
+    <t>LOJI AIR TRINGKAP</t>
+  </si>
+  <si>
+    <t>W1547948</t>
+  </si>
+  <si>
+    <t>CCHL/PCEJ00209</t>
+  </si>
+  <si>
+    <t>PAM PENGGALAK K.TERLA</t>
+  </si>
+  <si>
+    <t>W1547967</t>
+  </si>
+  <si>
+    <t>CCHL/PCEJ00238</t>
+  </si>
+  <si>
+    <t>ORIENTEL LILY</t>
+  </si>
+  <si>
+    <t>W1547997</t>
+  </si>
+  <si>
+    <t>CCHL/PCEJ00281</t>
+  </si>
+  <si>
+    <t>PE TMN PUNCAK TERLA</t>
+  </si>
+  <si>
+    <t>W1547893</t>
+  </si>
+  <si>
+    <t>CCHL/PCEJ00109</t>
+  </si>
+  <si>
+    <t>GUNUNG BRINCHANG</t>
+  </si>
+  <si>
+    <t>W1547894</t>
+  </si>
+  <si>
+    <t>CCHL/PCEJ00111</t>
+  </si>
+  <si>
+    <t>SG.PALAS LAB LINE</t>
+  </si>
+  <si>
+    <t>W1547895</t>
+  </si>
+  <si>
+    <t>CCHL/PCEJ00113</t>
+  </si>
+  <si>
+    <t>GERAK SEPADU</t>
+  </si>
+  <si>
+    <t>W1547896</t>
+  </si>
+  <si>
+    <t>CCHL/PCEJ00115</t>
+  </si>
+  <si>
+    <t>SG.PALAS FACTORY</t>
+  </si>
+  <si>
+    <t>W1547901</t>
+  </si>
+  <si>
+    <t>CCHL/PCEJ00120</t>
+  </si>
+  <si>
+    <t>K.Y KEONG</t>
+  </si>
+  <si>
+    <t>W1547989</t>
+  </si>
+  <si>
+    <t>CCHL/PCEJ00268</t>
+  </si>
+  <si>
+    <t>PALAS HORIZON</t>
+  </si>
+  <si>
+    <t>W1547990</t>
+  </si>
+  <si>
+    <t>CCHL/PCEJ00270</t>
+  </si>
+  <si>
+    <t>PALAS HORIZON APARTMENT</t>
+  </si>
+  <si>
+    <t>W1547996</t>
+  </si>
+  <si>
+    <t>CCHL/PCEJ00279</t>
+  </si>
+  <si>
+    <t>PE MOSSY FOREST</t>
   </si>
 </sst>
 </file>
@@ -477,314 +1395,1227 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" t="s">
+        <v>12</v>
+      </c>
       <c r="F2" s="2"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" t="s">
+        <v>15</v>
+      </c>
       <c r="F3" s="2"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" t="s">
+        <v>18</v>
+      </c>
       <c r="F4" s="2"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" t="s">
+        <v>21</v>
+      </c>
       <c r="F5" s="2"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" t="s">
+        <v>24</v>
+      </c>
       <c r="F6" s="2"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>25</v>
+      </c>
+      <c r="B7" t="s">
+        <v>26</v>
+      </c>
+      <c r="C7" t="s">
+        <v>27</v>
+      </c>
       <c r="F7" s="2"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" t="s">
+        <v>30</v>
+      </c>
       <c r="F8" s="2"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9" t="s">
+        <v>33</v>
+      </c>
       <c r="F9" s="2"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>34</v>
+      </c>
+      <c r="B10" t="s">
+        <v>35</v>
+      </c>
+      <c r="C10" t="s">
+        <v>36</v>
+      </c>
       <c r="F10" s="2"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>37</v>
+      </c>
+      <c r="B11" t="s">
+        <v>38</v>
+      </c>
+      <c r="C11" t="s">
+        <v>39</v>
+      </c>
       <c r="F11" s="2"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>40</v>
+      </c>
+      <c r="B12" t="s">
+        <v>41</v>
+      </c>
+      <c r="C12" t="s">
+        <v>42</v>
+      </c>
       <c r="F12" s="2"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>43</v>
+      </c>
+      <c r="B13" t="s">
+        <v>44</v>
+      </c>
+      <c r="C13" t="s">
+        <v>45</v>
+      </c>
       <c r="F13" s="2"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>46</v>
+      </c>
+      <c r="B14" t="s">
+        <v>47</v>
+      </c>
+      <c r="C14" t="s">
+        <v>48</v>
+      </c>
       <c r="F14" s="2"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>49</v>
+      </c>
+      <c r="B15" t="s">
+        <v>50</v>
+      </c>
+      <c r="C15" t="s">
+        <v>51</v>
+      </c>
       <c r="F15" s="2"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>52</v>
+      </c>
+      <c r="B16" t="s">
+        <v>53</v>
+      </c>
+      <c r="C16" t="s">
+        <v>54</v>
+      </c>
       <c r="F16" s="2"/>
     </row>
-    <row r="17" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>55</v>
+      </c>
+      <c r="B17" t="s">
+        <v>56</v>
+      </c>
+      <c r="C17" t="s">
+        <v>57</v>
+      </c>
       <c r="F17" s="2"/>
     </row>
-    <row r="18" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>58</v>
+      </c>
+      <c r="B18" t="s">
+        <v>59</v>
+      </c>
+      <c r="C18" t="s">
+        <v>60</v>
+      </c>
       <c r="F18" s="2"/>
     </row>
-    <row r="19" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>61</v>
+      </c>
+      <c r="B19" t="s">
+        <v>62</v>
+      </c>
+      <c r="C19" t="s">
+        <v>63</v>
+      </c>
       <c r="F19" s="2"/>
     </row>
-    <row r="20" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>64</v>
+      </c>
+      <c r="B20" t="s">
+        <v>65</v>
+      </c>
+      <c r="C20" t="s">
+        <v>66</v>
+      </c>
       <c r="F20" s="2"/>
     </row>
-    <row r="21" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>67</v>
+      </c>
+      <c r="B21" t="s">
+        <v>68</v>
+      </c>
+      <c r="C21" t="s">
+        <v>69</v>
+      </c>
       <c r="F21" s="2"/>
     </row>
-    <row r="22" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>70</v>
+      </c>
+      <c r="B22" t="s">
+        <v>71</v>
+      </c>
+      <c r="C22" t="s">
+        <v>72</v>
+      </c>
       <c r="F22" s="2"/>
     </row>
-    <row r="23" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>73</v>
+      </c>
+      <c r="B23" t="s">
+        <v>74</v>
+      </c>
+      <c r="C23" t="s">
+        <v>75</v>
+      </c>
       <c r="F23" s="2"/>
     </row>
-    <row r="24" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>76</v>
+      </c>
+      <c r="B24" t="s">
+        <v>77</v>
+      </c>
+      <c r="C24" t="s">
+        <v>78</v>
+      </c>
       <c r="F24" s="2"/>
     </row>
-    <row r="25" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>79</v>
+      </c>
+      <c r="B25" t="s">
+        <v>80</v>
+      </c>
+      <c r="C25" t="s">
+        <v>81</v>
+      </c>
       <c r="F25" s="2"/>
     </row>
-    <row r="26" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>82</v>
+      </c>
+      <c r="B26" t="s">
+        <v>83</v>
+      </c>
+      <c r="C26" t="s">
+        <v>84</v>
+      </c>
       <c r="F26" s="2"/>
     </row>
-    <row r="27" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>85</v>
+      </c>
+      <c r="B27" t="s">
+        <v>86</v>
+      </c>
+      <c r="C27" t="s">
+        <v>87</v>
+      </c>
       <c r="F27" s="2"/>
     </row>
-    <row r="28" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>88</v>
+      </c>
+      <c r="B28" t="s">
+        <v>89</v>
+      </c>
+      <c r="C28" t="s">
+        <v>90</v>
+      </c>
       <c r="F28" s="3"/>
     </row>
-    <row r="29" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>91</v>
+      </c>
+      <c r="B29" t="s">
+        <v>92</v>
+      </c>
+      <c r="C29" t="s">
+        <v>93</v>
+      </c>
       <c r="F29" s="3"/>
     </row>
-    <row r="30" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>94</v>
+      </c>
+      <c r="B30" t="s">
+        <v>95</v>
+      </c>
+      <c r="C30" t="s">
+        <v>96</v>
+      </c>
       <c r="F30" s="3"/>
     </row>
-    <row r="31" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>97</v>
+      </c>
+      <c r="B31" t="s">
+        <v>98</v>
+      </c>
+      <c r="C31" t="s">
+        <v>99</v>
+      </c>
       <c r="F31" s="3"/>
     </row>
-    <row r="32" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>100</v>
+      </c>
+      <c r="B32" t="s">
+        <v>101</v>
+      </c>
+      <c r="C32" t="s">
+        <v>102</v>
+      </c>
       <c r="F32" s="3"/>
     </row>
-    <row r="33" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>103</v>
+      </c>
+      <c r="B33" t="s">
+        <v>104</v>
+      </c>
+      <c r="C33" t="s">
+        <v>105</v>
+      </c>
       <c r="F33" s="3"/>
     </row>
-    <row r="34" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>106</v>
+      </c>
+      <c r="B34" t="s">
+        <v>107</v>
+      </c>
+      <c r="C34" t="s">
+        <v>108</v>
+      </c>
       <c r="F34" s="3"/>
     </row>
-    <row r="35" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>109</v>
+      </c>
+      <c r="B35" t="s">
+        <v>110</v>
+      </c>
+      <c r="C35" t="s">
+        <v>111</v>
+      </c>
       <c r="F35" s="3"/>
     </row>
-    <row r="36" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>112</v>
+      </c>
+      <c r="B36" t="s">
+        <v>113</v>
+      </c>
+      <c r="C36" t="s">
+        <v>114</v>
+      </c>
       <c r="F36" s="3"/>
     </row>
-    <row r="37" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>115</v>
+      </c>
+      <c r="B37" t="s">
+        <v>116</v>
+      </c>
+      <c r="C37" t="s">
+        <v>117</v>
+      </c>
       <c r="F37" s="3"/>
     </row>
-    <row r="38" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>118</v>
+      </c>
+      <c r="B38" t="s">
+        <v>119</v>
+      </c>
+      <c r="C38" t="s">
+        <v>120</v>
+      </c>
       <c r="F38" s="3"/>
     </row>
-    <row r="39" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>121</v>
+      </c>
+      <c r="B39" t="s">
+        <v>122</v>
+      </c>
+      <c r="C39" t="s">
+        <v>123</v>
+      </c>
       <c r="F39" s="3"/>
     </row>
-    <row r="40" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>124</v>
+      </c>
+      <c r="B40" t="s">
+        <v>125</v>
+      </c>
+      <c r="C40" t="s">
+        <v>126</v>
+      </c>
       <c r="F40" s="3"/>
     </row>
-    <row r="41" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>127</v>
+      </c>
+      <c r="B41" t="s">
+        <v>128</v>
+      </c>
+      <c r="C41" t="s">
+        <v>129</v>
+      </c>
       <c r="F41" s="3"/>
     </row>
-    <row r="42" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>130</v>
+      </c>
+      <c r="B42" t="s">
+        <v>131</v>
+      </c>
+      <c r="C42" t="s">
+        <v>132</v>
+      </c>
       <c r="F42" s="3"/>
     </row>
-    <row r="43" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>133</v>
+      </c>
+      <c r="B43" t="s">
+        <v>134</v>
+      </c>
+      <c r="C43" t="s">
+        <v>135</v>
+      </c>
       <c r="F43" s="3"/>
     </row>
-    <row r="44" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>136</v>
+      </c>
+      <c r="B44" t="s">
+        <v>137</v>
+      </c>
+      <c r="C44" t="s">
+        <v>138</v>
+      </c>
       <c r="F44" s="3"/>
     </row>
-    <row r="45" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>139</v>
+      </c>
+      <c r="B45" t="s">
+        <v>140</v>
+      </c>
+      <c r="C45" t="s">
+        <v>141</v>
+      </c>
       <c r="F45" s="3"/>
     </row>
-    <row r="46" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>142</v>
+      </c>
+      <c r="B46" t="s">
+        <v>143</v>
+      </c>
+      <c r="C46" t="s">
+        <v>144</v>
+      </c>
       <c r="F46" s="2"/>
     </row>
-    <row r="47" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>145</v>
+      </c>
+      <c r="B47" t="s">
+        <v>146</v>
+      </c>
+      <c r="C47" t="s">
+        <v>147</v>
+      </c>
       <c r="F47" s="3"/>
     </row>
-    <row r="48" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>148</v>
+      </c>
+      <c r="B48" t="s">
+        <v>149</v>
+      </c>
+      <c r="C48" t="s">
+        <v>150</v>
+      </c>
       <c r="F48" s="3"/>
     </row>
-    <row r="49" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>151</v>
+      </c>
+      <c r="B49" t="s">
+        <v>152</v>
+      </c>
+      <c r="C49" t="s">
+        <v>153</v>
+      </c>
       <c r="F49" s="3"/>
     </row>
-    <row r="50" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>154</v>
+      </c>
+      <c r="B50" t="s">
+        <v>155</v>
+      </c>
+      <c r="C50" t="s">
+        <v>156</v>
+      </c>
       <c r="F50" s="3"/>
     </row>
-    <row r="51" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>157</v>
+      </c>
+      <c r="B51" t="s">
+        <v>158</v>
+      </c>
+      <c r="C51" t="s">
+        <v>159</v>
+      </c>
       <c r="F51" s="3"/>
     </row>
-    <row r="52" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>160</v>
+      </c>
+      <c r="B52" t="s">
+        <v>161</v>
+      </c>
+      <c r="C52" t="s">
+        <v>162</v>
+      </c>
       <c r="F52" s="3"/>
     </row>
-    <row r="53" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>163</v>
+      </c>
+      <c r="B53" t="s">
+        <v>164</v>
+      </c>
+      <c r="C53" t="s">
+        <v>165</v>
+      </c>
       <c r="F53" s="3"/>
     </row>
-    <row r="54" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>166</v>
+      </c>
+      <c r="B54" t="s">
+        <v>167</v>
+      </c>
+      <c r="C54" t="s">
+        <v>168</v>
+      </c>
       <c r="F54" s="3"/>
     </row>
-    <row r="55" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>169</v>
+      </c>
+      <c r="B55" t="s">
+        <v>170</v>
+      </c>
+      <c r="C55" t="s">
+        <v>171</v>
+      </c>
       <c r="F55" s="3"/>
     </row>
-    <row r="56" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>172</v>
+      </c>
+      <c r="B56" t="s">
+        <v>173</v>
+      </c>
+      <c r="C56" t="s">
+        <v>174</v>
+      </c>
       <c r="F56" s="3"/>
     </row>
-    <row r="57" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>175</v>
+      </c>
+      <c r="B57" t="s">
+        <v>176</v>
+      </c>
+      <c r="C57" t="s">
+        <v>177</v>
+      </c>
       <c r="F57" s="3"/>
     </row>
-    <row r="58" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>178</v>
+      </c>
+      <c r="B58" t="s">
+        <v>179</v>
+      </c>
+      <c r="C58" t="s">
+        <v>180</v>
+      </c>
       <c r="F58" s="3"/>
     </row>
-    <row r="59" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>181</v>
+      </c>
+      <c r="B59" t="s">
+        <v>182</v>
+      </c>
+      <c r="C59" t="s">
+        <v>183</v>
+      </c>
       <c r="F59" s="3"/>
     </row>
-    <row r="60" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>184</v>
+      </c>
+      <c r="B60" t="s">
+        <v>185</v>
+      </c>
+      <c r="C60" t="s">
+        <v>186</v>
+      </c>
       <c r="F60" s="3"/>
     </row>
-    <row r="61" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>187</v>
+      </c>
+      <c r="B61" t="s">
+        <v>188</v>
+      </c>
+      <c r="C61" t="s">
+        <v>189</v>
+      </c>
       <c r="F61" s="3"/>
     </row>
-    <row r="62" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>190</v>
+      </c>
+      <c r="B62" t="s">
+        <v>191</v>
+      </c>
+      <c r="C62" t="s">
+        <v>192</v>
+      </c>
       <c r="F62" s="3"/>
     </row>
-    <row r="63" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>193</v>
+      </c>
+      <c r="B63" t="s">
+        <v>194</v>
+      </c>
+      <c r="C63" t="s">
+        <v>195</v>
+      </c>
       <c r="F63" s="3"/>
     </row>
-    <row r="64" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>196</v>
+      </c>
+      <c r="B64" t="s">
+        <v>197</v>
+      </c>
+      <c r="C64" t="s">
+        <v>198</v>
+      </c>
       <c r="F64" s="3"/>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>199</v>
+      </c>
+      <c r="B65" t="s">
+        <v>200</v>
+      </c>
+      <c r="C65" t="s">
+        <v>201</v>
+      </c>
       <c r="F65" s="3"/>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>202</v>
+      </c>
+      <c r="B66" t="s">
+        <v>203</v>
+      </c>
+      <c r="C66" t="s">
+        <v>204</v>
+      </c>
       <c r="F66" s="3"/>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>205</v>
+      </c>
+      <c r="B67" t="s">
+        <v>206</v>
+      </c>
+      <c r="C67" t="s">
+        <v>207</v>
+      </c>
       <c r="F67" s="3"/>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>208</v>
+      </c>
+      <c r="B68" t="s">
+        <v>209</v>
+      </c>
+      <c r="C68" t="s">
+        <v>210</v>
+      </c>
       <c r="F68" s="3"/>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>211</v>
+      </c>
+      <c r="B69" t="s">
+        <v>212</v>
+      </c>
+      <c r="C69" t="s">
+        <v>213</v>
+      </c>
       <c r="F69" s="3"/>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>214</v>
+      </c>
+      <c r="B70" t="s">
+        <v>215</v>
+      </c>
+      <c r="C70" t="s">
+        <v>216</v>
+      </c>
       <c r="F70" s="3"/>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A71" s="4"/>
+      <c r="A71" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="B71" t="s">
+        <v>218</v>
+      </c>
+      <c r="C71" t="s">
+        <v>219</v>
+      </c>
       <c r="F71" s="3"/>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A72" s="4"/>
+      <c r="A72" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="B72" t="s">
+        <v>221</v>
+      </c>
+      <c r="C72" t="s">
+        <v>222</v>
+      </c>
       <c r="F72" s="3"/>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A73" s="4"/>
+      <c r="A73" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="B73" t="s">
+        <v>224</v>
+      </c>
+      <c r="C73" t="s">
+        <v>225</v>
+      </c>
       <c r="F73" s="3"/>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A74" s="4"/>
+      <c r="A74" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="B74" t="s">
+        <v>227</v>
+      </c>
+      <c r="C74" t="s">
+        <v>228</v>
+      </c>
       <c r="F74" s="3"/>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A75" s="4"/>
+      <c r="A75" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="B75" t="s">
+        <v>230</v>
+      </c>
+      <c r="C75" t="s">
+        <v>231</v>
+      </c>
       <c r="F75" s="3"/>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>232</v>
+      </c>
+      <c r="B76" t="s">
+        <v>233</v>
+      </c>
+      <c r="C76" t="s">
+        <v>234</v>
+      </c>
       <c r="F76" s="3"/>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>235</v>
+      </c>
+      <c r="B77" t="s">
+        <v>236</v>
+      </c>
+      <c r="C77" t="s">
+        <v>237</v>
+      </c>
       <c r="F77" s="3"/>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>238</v>
+      </c>
+      <c r="B78" t="s">
+        <v>239</v>
+      </c>
+      <c r="C78" t="s">
+        <v>240</v>
+      </c>
       <c r="F78" s="2"/>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>241</v>
+      </c>
+      <c r="B79" t="s">
+        <v>242</v>
+      </c>
+      <c r="C79" t="s">
+        <v>243</v>
+      </c>
       <c r="F79" s="2"/>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>244</v>
+      </c>
+      <c r="B80" t="s">
+        <v>245</v>
+      </c>
+      <c r="C80" t="s">
+        <v>246</v>
+      </c>
       <c r="F80" s="2"/>
     </row>
-    <row r="81" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>247</v>
+      </c>
+      <c r="B81" t="s">
+        <v>248</v>
+      </c>
+      <c r="C81" t="s">
+        <v>249</v>
+      </c>
       <c r="F81" s="2"/>
     </row>
-    <row r="82" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>250</v>
+      </c>
+      <c r="B82" t="s">
+        <v>251</v>
+      </c>
+      <c r="C82" t="s">
+        <v>252</v>
+      </c>
       <c r="F82" s="2"/>
     </row>
-    <row r="83" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>253</v>
+      </c>
+      <c r="B83" t="s">
+        <v>254</v>
+      </c>
+      <c r="C83" t="s">
+        <v>255</v>
+      </c>
       <c r="F83" s="2"/>
     </row>
-    <row r="84" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>256</v>
+      </c>
+      <c r="B84" t="s">
+        <v>257</v>
+      </c>
+      <c r="C84" t="s">
+        <v>258</v>
+      </c>
       <c r="F84" s="2"/>
     </row>
-    <row r="85" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>259</v>
+      </c>
+      <c r="B85" t="s">
+        <v>260</v>
+      </c>
+      <c r="C85" t="s">
+        <v>261</v>
+      </c>
       <c r="F85" s="2"/>
     </row>
-    <row r="86" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>262</v>
+      </c>
+      <c r="B86" t="s">
+        <v>263</v>
+      </c>
+      <c r="C86" t="s">
+        <v>264</v>
+      </c>
       <c r="F86" s="2"/>
     </row>
-    <row r="87" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>265</v>
+      </c>
+      <c r="B87" t="s">
+        <v>266</v>
+      </c>
+      <c r="C87" t="s">
+        <v>267</v>
+      </c>
       <c r="F87" s="2"/>
     </row>
-    <row r="88" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>268</v>
+      </c>
+      <c r="B88" t="s">
+        <v>269</v>
+      </c>
+      <c r="C88" t="s">
+        <v>270</v>
+      </c>
       <c r="F88" s="2"/>
     </row>
-    <row r="89" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>271</v>
+      </c>
+      <c r="B89" t="s">
+        <v>272</v>
+      </c>
+      <c r="C89" t="s">
+        <v>273</v>
+      </c>
       <c r="F89" s="2"/>
     </row>
-    <row r="90" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>274</v>
+      </c>
+      <c r="B90" t="s">
+        <v>275</v>
+      </c>
+      <c r="C90" t="s">
+        <v>276</v>
+      </c>
       <c r="F90" s="2"/>
     </row>
-    <row r="91" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>277</v>
+      </c>
+      <c r="B91" t="s">
+        <v>278</v>
+      </c>
+      <c r="C91" t="s">
+        <v>279</v>
+      </c>
       <c r="F91" s="2"/>
     </row>
-    <row r="92" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>280</v>
+      </c>
+      <c r="B92" t="s">
+        <v>281</v>
+      </c>
+      <c r="C92" t="s">
+        <v>282</v>
+      </c>
       <c r="F92" s="2"/>
     </row>
-    <row r="93" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>283</v>
+      </c>
+      <c r="B93" t="s">
+        <v>284</v>
+      </c>
+      <c r="C93" t="s">
+        <v>285</v>
+      </c>
       <c r="F93" s="2"/>
     </row>
-    <row r="94" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>286</v>
+      </c>
+      <c r="B94" t="s">
+        <v>287</v>
+      </c>
+      <c r="C94" t="s">
+        <v>288</v>
+      </c>
       <c r="F94" s="2"/>
     </row>
-    <row r="95" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>289</v>
+      </c>
+      <c r="B95" t="s">
+        <v>290</v>
+      </c>
+      <c r="C95" t="s">
+        <v>291</v>
+      </c>
       <c r="F95" s="2"/>
     </row>
-    <row r="96" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>292</v>
+      </c>
+      <c r="B96" t="s">
+        <v>293</v>
+      </c>
+      <c r="C96" t="s">
+        <v>294</v>
+      </c>
       <c r="F96" s="2"/>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>295</v>
+      </c>
+      <c r="B97" t="s">
+        <v>296</v>
+      </c>
+      <c r="C97" t="s">
+        <v>297</v>
+      </c>
       <c r="F97" s="2"/>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>298</v>
+      </c>
+      <c r="B98" t="s">
+        <v>299</v>
+      </c>
+      <c r="C98" t="s">
+        <v>300</v>
+      </c>
       <c r="F98" s="2"/>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>301</v>
+      </c>
+      <c r="B99" t="s">
+        <v>302</v>
+      </c>
+      <c r="C99" t="s">
+        <v>303</v>
+      </c>
       <c r="F99" s="2"/>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>304</v>
+      </c>
+      <c r="B100" t="s">
+        <v>305</v>
+      </c>
+      <c r="C100" t="s">
+        <v>306</v>
+      </c>
       <c r="F100" s="2"/>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>307</v>
+      </c>
+      <c r="B101" t="s">
+        <v>308</v>
+      </c>
+      <c r="C101" t="s">
+        <v>309</v>
+      </c>
       <c r="F101" s="2"/>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>310</v>
+      </c>
+      <c r="B102" t="s">
+        <v>311</v>
+      </c>
+      <c r="C102" t="s">
+        <v>312</v>
+      </c>
       <c r="F102" s="2"/>
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>313</v>
+      </c>
+      <c r="B103" t="s">
+        <v>314</v>
+      </c>
+      <c r="C103" t="s">
+        <v>315</v>
+      </c>
       <c r="F103" s="2"/>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.25">

</xml_diff>